<commit_message>
updating documents, esp working on some final figs
</commit_message>
<xml_diff>
--- a/project_documents/parameterDirectory.xlsx
+++ b/project_documents/parameterDirectory.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/fabian/Documents/DPhil Work/Academic Work/EnglandCervicalScreeningProject/project_documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49999327-44F8-EB4B-A3A4-71A100E49CA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2C33E43B-BB4E-E745-9304-EAD4D6D39805}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="29400" windowHeight="17180" activeTab="7" xr2:uid="{9CDCC384-B02C-4946-8A51-C0AA91FF93D1}"/>
   </bookViews>
@@ -2146,7 +2146,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="43" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="318">
+  <cellXfs count="316">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -2587,12 +2587,6 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="11" fillId="6" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2600,8 +2594,11 @@
     <xf numFmtId="0" fontId="5" fillId="6" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="51" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2611,45 +2608,27 @@
     <xf numFmtId="0" fontId="10" fillId="0" borderId="66" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="2" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="6" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="29" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -2689,6 +2668,63 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="49" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -2731,63 +2767,6 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="20" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="8" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="24" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="9" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="21" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="8" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2801,23 +2780,86 @@
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="43" fontId="2" fillId="2" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="43" fontId="2" fillId="2" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="2" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="62" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="56" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="65" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
@@ -2839,82 +2881,38 @@
     <xf numFmtId="0" fontId="4" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="7" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="52" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="53" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="11" fillId="6" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="58" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="54" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="6" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="57" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="55" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="10" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="58" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="53" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="61" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="59" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="60" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="43" fontId="2" fillId="2" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="43" fontId="2" fillId="2" borderId="30" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="51" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="66" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="50" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Comma" xfId="1" builtinId="3"/>
@@ -3363,11 +3361,11 @@
       </c>
     </row>
     <row r="4" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B4" s="227" t="s">
+      <c r="B4" s="220" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="227"/>
-      <c r="D4" s="227"/>
+      <c r="C4" s="220"/>
+      <c r="D4" s="220"/>
     </row>
     <row r="5" spans="2:4" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B5" s="9" t="s">
@@ -3445,26 +3443,26 @@
       </c>
     </row>
     <row r="13" spans="2:4" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="228" t="s">
+      <c r="B13" s="221" t="s">
         <v>89</v>
       </c>
-      <c r="C13" s="228"/>
-      <c r="D13" s="228"/>
+      <c r="C13" s="221"/>
+      <c r="D13" s="221"/>
     </row>
     <row r="14" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B14" s="228"/>
-      <c r="C14" s="228"/>
-      <c r="D14" s="228"/>
+      <c r="B14" s="221"/>
+      <c r="C14" s="221"/>
+      <c r="D14" s="221"/>
     </row>
     <row r="15" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B15" s="228"/>
-      <c r="C15" s="228"/>
-      <c r="D15" s="228"/>
+      <c r="B15" s="221"/>
+      <c r="C15" s="221"/>
+      <c r="D15" s="221"/>
     </row>
     <row r="16" spans="2:4" x14ac:dyDescent="0.2">
-      <c r="B16" s="228"/>
-      <c r="C16" s="228"/>
-      <c r="D16" s="228"/>
+      <c r="B16" s="221"/>
+      <c r="C16" s="221"/>
+      <c r="D16" s="221"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3495,13 +3493,13 @@
       </c>
     </row>
     <row r="3" spans="2:6" ht="50" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="231" t="s">
+      <c r="B3" s="224" t="s">
         <v>229</v>
       </c>
-      <c r="C3" s="231"/>
-      <c r="D3" s="231"/>
-      <c r="E3" s="231"/>
-      <c r="F3" s="231"/>
+      <c r="C3" s="224"/>
+      <c r="D3" s="224"/>
+      <c r="E3" s="224"/>
+      <c r="F3" s="224"/>
     </row>
     <row r="5" spans="2:6" ht="35" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B5" s="19" t="s">
@@ -3521,7 +3519,7 @@
       </c>
     </row>
     <row r="6" spans="2:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="B6" s="233" t="s">
+      <c r="B6" s="226" t="s">
         <v>177</v>
       </c>
       <c r="C6" s="27" t="s">
@@ -3536,7 +3534,7 @@
       <c r="F6" s="14"/>
     </row>
     <row r="7" spans="2:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="B7" s="234"/>
+      <c r="B7" s="227"/>
       <c r="C7" s="28" t="s">
         <v>179</v>
       </c>
@@ -3549,7 +3547,7 @@
       <c r="F7" s="15"/>
     </row>
     <row r="8" spans="2:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="B8" s="234"/>
+      <c r="B8" s="227"/>
       <c r="C8" s="28" t="s">
         <v>180</v>
       </c>
@@ -3562,7 +3560,7 @@
       <c r="F8" s="15"/>
     </row>
     <row r="9" spans="2:6" ht="51" x14ac:dyDescent="0.2">
-      <c r="B9" s="234"/>
+      <c r="B9" s="227"/>
       <c r="C9" s="28" t="s">
         <v>181</v>
       </c>
@@ -3575,7 +3573,7 @@
       <c r="F9" s="15"/>
     </row>
     <row r="10" spans="2:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="B10" s="235" t="s">
+      <c r="B10" s="228" t="s">
         <v>173</v>
       </c>
       <c r="C10" s="29" t="s">
@@ -3592,7 +3590,7 @@
       </c>
     </row>
     <row r="11" spans="2:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="B11" s="235"/>
+      <c r="B11" s="228"/>
       <c r="C11" s="29" t="s">
         <v>187</v>
       </c>
@@ -3607,7 +3605,7 @@
       </c>
     </row>
     <row r="12" spans="2:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="B12" s="235"/>
+      <c r="B12" s="228"/>
       <c r="C12" s="29" t="s">
         <v>188</v>
       </c>
@@ -3622,7 +3620,7 @@
       </c>
     </row>
     <row r="13" spans="2:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="B13" s="236" t="s">
+      <c r="B13" s="229" t="s">
         <v>174</v>
       </c>
       <c r="C13" s="30" t="s">
@@ -3639,7 +3637,7 @@
       </c>
     </row>
     <row r="14" spans="2:6" ht="34" x14ac:dyDescent="0.2">
-      <c r="B14" s="236"/>
+      <c r="B14" s="229"/>
       <c r="C14" s="30" t="s">
         <v>113</v>
       </c>
@@ -3654,7 +3652,7 @@
       </c>
     </row>
     <row r="15" spans="2:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="B15" s="236"/>
+      <c r="B15" s="229"/>
       <c r="C15" s="30" t="s">
         <v>111</v>
       </c>
@@ -3669,7 +3667,7 @@
       </c>
     </row>
     <row r="16" spans="2:6" ht="17" x14ac:dyDescent="0.2">
-      <c r="B16" s="237" t="s">
+      <c r="B16" s="230" t="s">
         <v>175</v>
       </c>
       <c r="C16" s="31" t="s">
@@ -3684,7 +3682,7 @@
       <c r="F16" s="18"/>
     </row>
     <row r="17" spans="2:11" ht="34" x14ac:dyDescent="0.2">
-      <c r="B17" s="237"/>
+      <c r="B17" s="230"/>
       <c r="C17" s="31" t="s">
         <v>133</v>
       </c>
@@ -3699,7 +3697,7 @@
       </c>
     </row>
     <row r="18" spans="2:11" ht="135" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B18" s="237"/>
+      <c r="B18" s="230"/>
       <c r="C18" s="31" t="s">
         <v>115</v>
       </c>
@@ -3721,7 +3719,7 @@
       <c r="K18" s="4"/>
     </row>
     <row r="19" spans="2:11" ht="34" x14ac:dyDescent="0.2">
-      <c r="B19" s="237"/>
+      <c r="B19" s="230"/>
       <c r="C19" s="31" t="s">
         <v>114</v>
       </c>
@@ -3740,30 +3738,30 @@
       <c r="F21" s="4"/>
     </row>
     <row r="22" spans="2:11" ht="17" x14ac:dyDescent="0.2">
-      <c r="B22" s="238" t="s">
+      <c r="B22" s="231" t="s">
         <v>132</v>
       </c>
       <c r="C22" s="37" t="s">
         <v>116</v>
       </c>
-      <c r="D22" s="229" t="s">
+      <c r="D22" s="222" t="s">
         <v>216</v>
       </c>
-      <c r="E22" s="230"/>
+      <c r="E22" s="223"/>
     </row>
     <row r="23" spans="2:11" ht="32" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B23" s="239"/>
+      <c r="B23" s="232"/>
       <c r="C23" s="8" t="s">
         <v>115</v>
       </c>
-      <c r="D23" s="231" t="s">
+      <c r="D23" s="224" t="s">
         <v>218</v>
       </c>
-      <c r="E23" s="232"/>
+      <c r="E23" s="225"/>
       <c r="F23" s="4"/>
     </row>
     <row r="24" spans="2:11" x14ac:dyDescent="0.2">
-      <c r="B24" s="239"/>
+      <c r="B24" s="232"/>
       <c r="C24" s="8" t="s">
         <v>114</v>
       </c>
@@ -3834,30 +3832,30 @@
   <sheetData>
     <row r="2" spans="1:10" s="66" customFormat="1" ht="16" x14ac:dyDescent="0.2">
       <c r="A2" s="188"/>
-      <c r="B2" s="260" t="s">
+      <c r="B2" s="233" t="s">
         <v>7</v>
       </c>
-      <c r="C2" s="264" t="s">
+      <c r="C2" s="237" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="270" t="s">
+      <c r="D2" s="245" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="271"/>
-      <c r="F2" s="272" t="s">
+      <c r="E2" s="246"/>
+      <c r="F2" s="247" t="s">
         <v>11</v>
       </c>
-      <c r="G2" s="272"/>
-      <c r="H2" s="272"/>
-      <c r="I2" s="271"/>
-      <c r="J2" s="262" t="s">
+      <c r="G2" s="247"/>
+      <c r="H2" s="247"/>
+      <c r="I2" s="246"/>
+      <c r="J2" s="235" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="3" spans="1:10" s="66" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="188"/>
-      <c r="B3" s="261"/>
-      <c r="C3" s="265"/>
+      <c r="B3" s="234"/>
+      <c r="C3" s="238"/>
       <c r="D3" s="11" t="s">
         <v>9</v>
       </c>
@@ -3876,10 +3874,10 @@
       <c r="I3" s="189" t="s">
         <v>25</v>
       </c>
-      <c r="J3" s="263"/>
+      <c r="J3" s="236"/>
     </row>
     <row r="4" spans="1:10" s="86" customFormat="1" ht="91" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="255" t="s">
+      <c r="A4" s="249" t="s">
         <v>85</v>
       </c>
       <c r="B4" s="81" t="s">
@@ -3903,7 +3901,7 @@
       </c>
     </row>
     <row r="5" spans="1:10" s="86" customFormat="1" ht="105" x14ac:dyDescent="0.2">
-      <c r="A5" s="255"/>
+      <c r="A5" s="249"/>
       <c r="B5" s="88" t="s">
         <v>18</v>
       </c>
@@ -3925,7 +3923,7 @@
       </c>
     </row>
     <row r="6" spans="1:10" s="86" customFormat="1" ht="60" x14ac:dyDescent="0.2">
-      <c r="A6" s="255"/>
+      <c r="A6" s="249"/>
       <c r="B6" s="88" t="s">
         <v>22</v>
       </c>
@@ -3945,7 +3943,7 @@
       <c r="J6" s="89"/>
     </row>
     <row r="7" spans="1:10" s="86" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A7" s="255"/>
+      <c r="A7" s="249"/>
       <c r="B7" s="88" t="s">
         <v>101</v>
       </c>
@@ -3965,7 +3963,7 @@
       <c r="J7" s="89"/>
     </row>
     <row r="8" spans="1:10" s="86" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A8" s="255"/>
+      <c r="A8" s="249"/>
       <c r="B8" s="88" t="s">
         <v>23</v>
       </c>
@@ -4009,7 +4007,7 @@
       </c>
     </row>
     <row r="10" spans="1:10" s="103" customFormat="1" ht="90" x14ac:dyDescent="0.2">
-      <c r="A10" s="256" t="s">
+      <c r="A10" s="250" t="s">
         <v>87</v>
       </c>
       <c r="B10" s="98" t="s">
@@ -4033,37 +4031,37 @@
       </c>
     </row>
     <row r="11" spans="1:10" s="103" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="256"/>
-      <c r="B11" s="258" t="s">
+      <c r="A11" s="250"/>
+      <c r="B11" s="241" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="266" t="s">
+      <c r="C11" s="239" t="s">
         <v>39</v>
       </c>
       <c r="D11" s="101"/>
-      <c r="E11" s="258" t="s">
+      <c r="E11" s="241" t="s">
         <v>327</v>
       </c>
       <c r="F11" s="101"/>
       <c r="G11" s="102"/>
       <c r="H11" s="102"/>
       <c r="I11" s="98"/>
-      <c r="J11" s="268"/>
+      <c r="J11" s="243"/>
     </row>
     <row r="12" spans="1:10" s="103" customFormat="1" ht="60" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="256"/>
-      <c r="B12" s="259"/>
-      <c r="C12" s="267"/>
+      <c r="A12" s="250"/>
+      <c r="B12" s="242"/>
+      <c r="C12" s="240"/>
       <c r="D12" s="101"/>
-      <c r="E12" s="259"/>
+      <c r="E12" s="242"/>
       <c r="F12" s="101"/>
       <c r="G12" s="102"/>
       <c r="H12" s="102"/>
       <c r="I12" s="98"/>
-      <c r="J12" s="269"/>
+      <c r="J12" s="244"/>
     </row>
     <row r="13" spans="1:10" s="108" customFormat="1" ht="105" x14ac:dyDescent="0.2">
-      <c r="A13" s="257" t="s">
+      <c r="A13" s="251" t="s">
         <v>88</v>
       </c>
       <c r="B13" s="104" t="s">
@@ -4085,7 +4083,7 @@
       <c r="J13" s="106"/>
     </row>
     <row r="14" spans="1:10" s="108" customFormat="1" ht="188" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="257"/>
+      <c r="A14" s="251"/>
       <c r="B14" s="104" t="s">
         <v>35</v>
       </c>
@@ -4107,7 +4105,7 @@
       </c>
     </row>
     <row r="15" spans="1:10" s="108" customFormat="1" ht="45" x14ac:dyDescent="0.2">
-      <c r="A15" s="257"/>
+      <c r="A15" s="251"/>
       <c r="B15" s="104" t="s">
         <v>44</v>
       </c>
@@ -4127,7 +4125,7 @@
       <c r="J15" s="106"/>
     </row>
     <row r="16" spans="1:10" s="108" customFormat="1" ht="60" x14ac:dyDescent="0.2">
-      <c r="A16" s="257"/>
+      <c r="A16" s="251"/>
       <c r="B16" s="104" t="s">
         <v>47</v>
       </c>
@@ -4149,7 +4147,7 @@
       </c>
     </row>
     <row r="17" spans="1:10" s="108" customFormat="1" ht="30" x14ac:dyDescent="0.2">
-      <c r="A17" s="257"/>
+      <c r="A17" s="251"/>
       <c r="B17" s="104" t="s">
         <v>51</v>
       </c>
@@ -4169,7 +4167,7 @@
       <c r="J17" s="106"/>
     </row>
     <row r="18" spans="1:10" s="108" customFormat="1" ht="135" x14ac:dyDescent="0.2">
-      <c r="A18" s="257"/>
+      <c r="A18" s="251"/>
       <c r="B18" s="104" t="s">
         <v>55</v>
       </c>
@@ -4193,7 +4191,7 @@
       <c r="J18" s="106"/>
     </row>
     <row r="19" spans="1:10" s="108" customFormat="1" ht="105" x14ac:dyDescent="0.2">
-      <c r="A19" s="257"/>
+      <c r="A19" s="251"/>
       <c r="B19" s="104" t="s">
         <v>58</v>
       </c>
@@ -4217,7 +4215,7 @@
       <c r="J19" s="106"/>
     </row>
     <row r="20" spans="1:10" s="108" customFormat="1" ht="115" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A20" s="257"/>
+      <c r="A20" s="251"/>
       <c r="B20" s="104" t="s">
         <v>61</v>
       </c>
@@ -4237,51 +4235,51 @@
       <c r="J20" s="110"/>
     </row>
     <row r="21" spans="1:10" s="43" customFormat="1" ht="120" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A21" s="257"/>
+      <c r="A21" s="251"/>
       <c r="B21" s="191" t="s">
         <v>95</v>
       </c>
-      <c r="C21" s="243" t="s">
+      <c r="C21" s="255" t="s">
         <v>98</v>
       </c>
       <c r="D21" s="110" t="s">
         <v>165</v>
       </c>
-      <c r="E21" s="240" t="s">
+      <c r="E21" s="252" t="s">
         <v>99</v>
       </c>
       <c r="F21" s="72"/>
       <c r="G21" s="73"/>
       <c r="H21" s="73"/>
-      <c r="I21" s="240" t="s">
+      <c r="I21" s="252" t="s">
         <v>167</v>
       </c>
-      <c r="J21" s="246" t="s">
+      <c r="J21" s="258" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="22" spans="1:10" s="43" customFormat="1" ht="52" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A22" s="257"/>
+      <c r="A22" s="251"/>
       <c r="B22" s="192" t="s">
         <v>97</v>
       </c>
-      <c r="C22" s="244"/>
+      <c r="C22" s="256"/>
       <c r="D22" s="193" t="s">
         <v>166</v>
       </c>
-      <c r="E22" s="241"/>
+      <c r="E22" s="253"/>
       <c r="F22" s="71"/>
       <c r="G22" s="69"/>
       <c r="H22" s="69"/>
-      <c r="I22" s="241"/>
-      <c r="J22" s="247"/>
+      <c r="I22" s="253"/>
+      <c r="J22" s="259"/>
     </row>
     <row r="23" spans="1:10" s="43" customFormat="1" ht="180" x14ac:dyDescent="0.2">
-      <c r="A23" s="257"/>
+      <c r="A23" s="251"/>
       <c r="B23" s="104" t="s">
         <v>96</v>
       </c>
-      <c r="C23" s="245"/>
+      <c r="C23" s="257"/>
       <c r="D23" s="110" t="s">
         <v>308</v>
       </c>
@@ -4291,8 +4289,8 @@
       <c r="F23" s="74"/>
       <c r="G23" s="69"/>
       <c r="H23" s="69"/>
-      <c r="I23" s="242"/>
-      <c r="J23" s="248"/>
+      <c r="I23" s="254"/>
+      <c r="J23" s="260"/>
     </row>
     <row r="24" spans="1:10" s="43" customFormat="1" ht="255" x14ac:dyDescent="0.2">
       <c r="A24" s="190"/>
@@ -4365,7 +4363,7 @@
       <c r="B27" s="120" t="s">
         <v>67</v>
       </c>
-      <c r="C27" s="251" t="s">
+      <c r="C27" s="263" t="s">
         <v>79</v>
       </c>
       <c r="D27" s="122"/>
@@ -4391,7 +4389,7 @@
       <c r="B28" s="120" t="s">
         <v>82</v>
       </c>
-      <c r="C28" s="252"/>
+      <c r="C28" s="264"/>
       <c r="D28" s="122">
         <v>50</v>
       </c>
@@ -4409,7 +4407,7 @@
       <c r="B29" s="120" t="s">
         <v>83</v>
       </c>
-      <c r="C29" s="253"/>
+      <c r="C29" s="265"/>
       <c r="D29" s="122">
         <v>0</v>
       </c>
@@ -4497,7 +4495,7 @@
       <c r="J32" s="122"/>
     </row>
     <row r="33" spans="1:10" s="132" customFormat="1" ht="180" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A33" s="254" t="s">
+      <c r="A33" s="248" t="s">
         <v>239</v>
       </c>
       <c r="B33" s="128" t="s">
@@ -4516,12 +4514,12 @@
       <c r="G33" s="131"/>
       <c r="H33" s="131"/>
       <c r="I33" s="128"/>
-      <c r="J33" s="249" t="s">
+      <c r="J33" s="261" t="s">
         <v>238</v>
       </c>
     </row>
     <row r="34" spans="1:10" s="132" customFormat="1" ht="60" x14ac:dyDescent="0.2">
-      <c r="A34" s="254"/>
+      <c r="A34" s="248"/>
       <c r="B34" s="128" t="s">
         <v>106</v>
       </c>
@@ -4538,10 +4536,21 @@
       <c r="G34" s="131"/>
       <c r="H34" s="131"/>
       <c r="I34" s="128"/>
-      <c r="J34" s="250"/>
+      <c r="J34" s="262"/>
     </row>
   </sheetData>
   <mergeCells count="19">
+    <mergeCell ref="I21:I23"/>
+    <mergeCell ref="C21:C23"/>
+    <mergeCell ref="E21:E22"/>
+    <mergeCell ref="J21:J23"/>
+    <mergeCell ref="J33:J34"/>
+    <mergeCell ref="C27:C29"/>
+    <mergeCell ref="A33:A34"/>
+    <mergeCell ref="A4:A8"/>
+    <mergeCell ref="A10:A12"/>
+    <mergeCell ref="A13:A23"/>
+    <mergeCell ref="B11:B12"/>
     <mergeCell ref="B2:B3"/>
     <mergeCell ref="J2:J3"/>
     <mergeCell ref="C2:C3"/>
@@ -4550,17 +4559,6 @@
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="D2:E2"/>
     <mergeCell ref="F2:I2"/>
-    <mergeCell ref="A33:A34"/>
-    <mergeCell ref="A4:A8"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="A13:A23"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="I21:I23"/>
-    <mergeCell ref="C21:C23"/>
-    <mergeCell ref="E21:E22"/>
-    <mergeCell ref="J21:J23"/>
-    <mergeCell ref="J33:J34"/>
-    <mergeCell ref="C27:C29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -4614,7 +4612,7 @@
       <c r="E2" s="158">
         <v>0.12</v>
       </c>
-      <c r="H2" s="273" t="s">
+      <c r="H2" s="266" t="s">
         <v>304</v>
       </c>
     </row>
@@ -4634,7 +4632,7 @@
       <c r="E3" s="162">
         <v>0.88</v>
       </c>
-      <c r="H3" s="273"/>
+      <c r="H3" s="266"/>
     </row>
     <row r="4" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A4" s="136" t="s">
@@ -4652,7 +4650,7 @@
       <c r="E4" s="162">
         <v>0</v>
       </c>
-      <c r="H4" s="273"/>
+      <c r="H4" s="266"/>
     </row>
     <row r="5" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A5" s="136" t="s">
@@ -4670,7 +4668,7 @@
       <c r="E5" s="158">
         <v>0.12</v>
       </c>
-      <c r="H5" s="273"/>
+      <c r="H5" s="266"/>
     </row>
     <row r="6" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A6" s="136" t="s">
@@ -4688,7 +4686,7 @@
       <c r="E6" s="162">
         <v>0.88</v>
       </c>
-      <c r="H6" s="273"/>
+      <c r="H6" s="266"/>
     </row>
     <row r="7" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A7" s="136" t="s">
@@ -4706,7 +4704,7 @@
       <c r="E7" s="162">
         <v>0</v>
       </c>
-      <c r="H7" s="273"/>
+      <c r="H7" s="266"/>
     </row>
     <row r="8" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A8" s="136" t="s">
@@ -4724,7 +4722,7 @@
       <c r="E8" s="158">
         <v>0.12</v>
       </c>
-      <c r="H8" s="273"/>
+      <c r="H8" s="266"/>
     </row>
     <row r="9" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A9" s="136" t="s">
@@ -4742,7 +4740,7 @@
       <c r="E9" s="162">
         <v>0.88</v>
       </c>
-      <c r="H9" s="273"/>
+      <c r="H9" s="266"/>
     </row>
     <row r="10" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A10" s="136" t="s">
@@ -4760,7 +4758,7 @@
       <c r="E10" s="162">
         <v>0</v>
       </c>
-      <c r="H10" s="273"/>
+      <c r="H10" s="266"/>
     </row>
     <row r="11" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A11" s="136" t="s">
@@ -4778,7 +4776,7 @@
       <c r="E11" s="158">
         <v>0.12</v>
       </c>
-      <c r="H11" s="273"/>
+      <c r="H11" s="266"/>
     </row>
     <row r="12" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A12" s="136" t="s">
@@ -4796,7 +4794,7 @@
       <c r="E12" s="162">
         <v>0.88</v>
       </c>
-      <c r="H12" s="273"/>
+      <c r="H12" s="266"/>
     </row>
     <row r="13" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A13" s="136" t="s">
@@ -4814,7 +4812,7 @@
       <c r="E13" s="162">
         <v>0</v>
       </c>
-      <c r="H13" s="273"/>
+      <c r="H13" s="266"/>
     </row>
     <row r="14" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A14" s="136" t="s">
@@ -4832,7 +4830,7 @@
       <c r="E14" s="158">
         <v>0.12</v>
       </c>
-      <c r="H14" s="273"/>
+      <c r="H14" s="266"/>
     </row>
     <row r="15" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A15" s="136" t="s">
@@ -4850,7 +4848,7 @@
       <c r="E15" s="162">
         <v>0.88</v>
       </c>
-      <c r="H15" s="273"/>
+      <c r="H15" s="266"/>
     </row>
     <row r="16" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A16" s="136" t="s">
@@ -4868,7 +4866,7 @@
       <c r="E16" s="162">
         <v>0</v>
       </c>
-      <c r="H16" s="273"/>
+      <c r="H16" s="266"/>
     </row>
     <row r="17" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A17" s="136" t="s">
@@ -4886,7 +4884,7 @@
       <c r="E17" s="158">
         <v>0.12</v>
       </c>
-      <c r="H17" s="273"/>
+      <c r="H17" s="266"/>
     </row>
     <row r="18" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A18" s="136" t="s">
@@ -4904,7 +4902,7 @@
       <c r="E18" s="162">
         <v>0.88</v>
       </c>
-      <c r="H18" s="273"/>
+      <c r="H18" s="266"/>
     </row>
     <row r="19" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A19" s="136" t="s">
@@ -4922,7 +4920,7 @@
       <c r="E19" s="162">
         <v>0</v>
       </c>
-      <c r="H19" s="273"/>
+      <c r="H19" s="266"/>
     </row>
     <row r="20" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A20" s="136" t="s">
@@ -4940,7 +4938,7 @@
       <c r="E20" s="158">
         <v>0.12</v>
       </c>
-      <c r="H20" s="273"/>
+      <c r="H20" s="266"/>
     </row>
     <row r="21" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A21" s="136" t="s">
@@ -4958,7 +4956,7 @@
       <c r="E21" s="162">
         <v>0.88</v>
       </c>
-      <c r="H21" s="273"/>
+      <c r="H21" s="266"/>
     </row>
     <row r="22" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A22" s="136" t="s">
@@ -4976,7 +4974,7 @@
       <c r="E22" s="162">
         <v>0</v>
       </c>
-      <c r="H22" s="273"/>
+      <c r="H22" s="266"/>
     </row>
     <row r="23" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A23" s="136" t="s">
@@ -4994,7 +4992,7 @@
       <c r="E23" s="158">
         <v>0.12</v>
       </c>
-      <c r="H23" s="273"/>
+      <c r="H23" s="266"/>
     </row>
     <row r="24" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A24" s="136" t="s">
@@ -5012,7 +5010,7 @@
       <c r="E24" s="162">
         <v>0.88</v>
       </c>
-      <c r="H24" s="273"/>
+      <c r="H24" s="266"/>
     </row>
     <row r="25" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A25" s="136" t="s">
@@ -5030,7 +5028,7 @@
       <c r="E25" s="162">
         <v>0</v>
       </c>
-      <c r="H25" s="273"/>
+      <c r="H25" s="266"/>
     </row>
     <row r="26" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A26" s="136" t="s">
@@ -5048,7 +5046,7 @@
       <c r="E26" s="158">
         <v>0.12</v>
       </c>
-      <c r="H26" s="273"/>
+      <c r="H26" s="266"/>
     </row>
     <row r="27" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A27" s="136" t="s">
@@ -5066,7 +5064,7 @@
       <c r="E27" s="162">
         <v>0.88</v>
       </c>
-      <c r="H27" s="273"/>
+      <c r="H27" s="266"/>
     </row>
     <row r="28" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A28" s="136" t="s">
@@ -5084,7 +5082,7 @@
       <c r="E28" s="162">
         <v>0</v>
       </c>
-      <c r="H28" s="273"/>
+      <c r="H28" s="266"/>
     </row>
     <row r="29" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A29" s="136" t="s">
@@ -5102,7 +5100,7 @@
       <c r="E29" s="158">
         <v>0.12</v>
       </c>
-      <c r="H29" s="273"/>
+      <c r="H29" s="266"/>
     </row>
     <row r="30" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A30" s="136" t="s">
@@ -5120,7 +5118,7 @@
       <c r="E30" s="162">
         <v>0.88</v>
       </c>
-      <c r="H30" s="273"/>
+      <c r="H30" s="266"/>
     </row>
     <row r="31" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A31" s="136" t="s">
@@ -5138,7 +5136,7 @@
       <c r="E31" s="162">
         <v>0</v>
       </c>
-      <c r="H31" s="273"/>
+      <c r="H31" s="266"/>
     </row>
     <row r="32" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A32" s="136" t="s">
@@ -5156,7 +5154,7 @@
       <c r="E32" s="158">
         <v>0.12</v>
       </c>
-      <c r="H32" s="273"/>
+      <c r="H32" s="266"/>
     </row>
     <row r="33" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A33" s="136" t="s">
@@ -5174,7 +5172,7 @@
       <c r="E33" s="162">
         <v>0.88</v>
       </c>
-      <c r="H33" s="273"/>
+      <c r="H33" s="266"/>
     </row>
     <row r="34" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A34" s="136" t="s">
@@ -5192,7 +5190,7 @@
       <c r="E34" s="162">
         <v>0</v>
       </c>
-      <c r="H34" s="273"/>
+      <c r="H34" s="266"/>
     </row>
     <row r="35" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A35" s="136" t="s">
@@ -5210,7 +5208,7 @@
       <c r="E35" s="158">
         <v>0.12</v>
       </c>
-      <c r="H35" s="273"/>
+      <c r="H35" s="266"/>
     </row>
     <row r="36" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A36" s="136" t="s">
@@ -5228,7 +5226,7 @@
       <c r="E36" s="162">
         <v>0.88</v>
       </c>
-      <c r="H36" s="273"/>
+      <c r="H36" s="266"/>
     </row>
     <row r="37" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A37" s="136" t="s">
@@ -5246,7 +5244,7 @@
       <c r="E37" s="162">
         <v>0</v>
       </c>
-      <c r="H37" s="273"/>
+      <c r="H37" s="266"/>
     </row>
     <row r="38" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A38" s="136" t="s">
@@ -5264,7 +5262,7 @@
       <c r="E38" s="162">
         <v>0.94</v>
       </c>
-      <c r="H38" s="273"/>
+      <c r="H38" s="266"/>
     </row>
     <row r="39" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A39" s="136" t="s">
@@ -5282,7 +5280,7 @@
       <c r="E39" s="162">
         <v>0.06</v>
       </c>
-      <c r="H39" s="273"/>
+      <c r="H39" s="266"/>
     </row>
     <row r="40" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A40" s="136" t="s">
@@ -5300,7 +5298,7 @@
       <c r="E40" s="162">
         <v>0</v>
       </c>
-      <c r="H40" s="273"/>
+      <c r="H40" s="266"/>
     </row>
     <row r="41" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A41" s="136" t="s">
@@ -5318,7 +5316,7 @@
       <c r="E41" s="162">
         <v>0.94</v>
       </c>
-      <c r="H41" s="273"/>
+      <c r="H41" s="266"/>
     </row>
     <row r="42" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A42" s="136" t="s">
@@ -5336,7 +5334,7 @@
       <c r="E42" s="162">
         <v>0.06</v>
       </c>
-      <c r="H42" s="273"/>
+      <c r="H42" s="266"/>
     </row>
     <row r="43" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A43" s="136" t="s">
@@ -5354,7 +5352,7 @@
       <c r="E43" s="162">
         <v>0</v>
       </c>
-      <c r="H43" s="273"/>
+      <c r="H43" s="266"/>
     </row>
     <row r="44" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A44" s="136" t="s">
@@ -5372,7 +5370,7 @@
       <c r="E44" s="162">
         <v>0.94</v>
       </c>
-      <c r="H44" s="273"/>
+      <c r="H44" s="266"/>
     </row>
     <row r="45" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A45" s="136" t="s">
@@ -5390,7 +5388,7 @@
       <c r="E45" s="162">
         <v>0.06</v>
       </c>
-      <c r="H45" s="273"/>
+      <c r="H45" s="266"/>
     </row>
     <row r="46" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A46" s="136" t="s">
@@ -5408,7 +5406,7 @@
       <c r="E46" s="162">
         <v>0</v>
       </c>
-      <c r="H46" s="273"/>
+      <c r="H46" s="266"/>
     </row>
     <row r="47" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A47" s="136" t="s">
@@ -5426,7 +5424,7 @@
       <c r="E47" s="162">
         <v>0.94</v>
       </c>
-      <c r="H47" s="273"/>
+      <c r="H47" s="266"/>
     </row>
     <row r="48" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A48" s="136" t="s">
@@ -5444,7 +5442,7 @@
       <c r="E48" s="162">
         <v>0.06</v>
       </c>
-      <c r="H48" s="273"/>
+      <c r="H48" s="266"/>
     </row>
     <row r="49" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A49" s="136" t="s">
@@ -5462,7 +5460,7 @@
       <c r="E49" s="162">
         <v>0</v>
       </c>
-      <c r="H49" s="273"/>
+      <c r="H49" s="266"/>
     </row>
     <row r="50" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A50" s="136" t="s">
@@ -5480,7 +5478,7 @@
       <c r="E50" s="162">
         <v>0.94</v>
       </c>
-      <c r="H50" s="273"/>
+      <c r="H50" s="266"/>
     </row>
     <row r="51" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A51" s="136" t="s">
@@ -5498,7 +5496,7 @@
       <c r="E51" s="162">
         <v>0.06</v>
       </c>
-      <c r="H51" s="273"/>
+      <c r="H51" s="266"/>
     </row>
     <row r="52" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A52" s="136" t="s">
@@ -5516,7 +5514,7 @@
       <c r="E52" s="162">
         <v>0</v>
       </c>
-      <c r="H52" s="273"/>
+      <c r="H52" s="266"/>
     </row>
     <row r="53" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A53" s="136" t="s">
@@ -5534,7 +5532,7 @@
       <c r="E53" s="162">
         <v>0.94</v>
       </c>
-      <c r="H53" s="273"/>
+      <c r="H53" s="266"/>
     </row>
     <row r="54" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A54" s="136" t="s">
@@ -5552,7 +5550,7 @@
       <c r="E54" s="162">
         <v>0.06</v>
       </c>
-      <c r="H54" s="273"/>
+      <c r="H54" s="266"/>
     </row>
     <row r="55" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A55" s="136" t="s">
@@ -5570,7 +5568,7 @@
       <c r="E55" s="162">
         <v>0</v>
       </c>
-      <c r="H55" s="273"/>
+      <c r="H55" s="266"/>
     </row>
     <row r="56" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A56" s="136" t="s">
@@ -5588,7 +5586,7 @@
       <c r="E56" s="162">
         <v>0.94</v>
       </c>
-      <c r="H56" s="273"/>
+      <c r="H56" s="266"/>
     </row>
     <row r="57" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A57" s="136" t="s">
@@ -5606,7 +5604,7 @@
       <c r="E57" s="162">
         <v>0.06</v>
       </c>
-      <c r="H57" s="273"/>
+      <c r="H57" s="266"/>
     </row>
     <row r="58" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A58" s="136" t="s">
@@ -5624,7 +5622,7 @@
       <c r="E58" s="162">
         <v>0</v>
       </c>
-      <c r="H58" s="273"/>
+      <c r="H58" s="266"/>
     </row>
     <row r="59" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A59" s="136" t="s">
@@ -5642,7 +5640,7 @@
       <c r="E59" s="162">
         <v>0.94</v>
       </c>
-      <c r="H59" s="273"/>
+      <c r="H59" s="266"/>
     </row>
     <row r="60" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A60" s="136" t="s">
@@ -5660,7 +5658,7 @@
       <c r="E60" s="162">
         <v>0.06</v>
       </c>
-      <c r="H60" s="273"/>
+      <c r="H60" s="266"/>
     </row>
     <row r="61" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A61" s="136" t="s">
@@ -5678,7 +5676,7 @@
       <c r="E61" s="162">
         <v>0</v>
       </c>
-      <c r="H61" s="273"/>
+      <c r="H61" s="266"/>
     </row>
     <row r="62" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A62" s="136" t="s">
@@ -5696,7 +5694,7 @@
       <c r="E62" s="162">
         <v>0.94</v>
       </c>
-      <c r="H62" s="273"/>
+      <c r="H62" s="266"/>
     </row>
     <row r="63" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A63" s="136" t="s">
@@ -5714,7 +5712,7 @@
       <c r="E63" s="162">
         <v>0.06</v>
       </c>
-      <c r="H63" s="273"/>
+      <c r="H63" s="266"/>
     </row>
     <row r="64" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A64" s="136" t="s">
@@ -5732,7 +5730,7 @@
       <c r="E64" s="162">
         <v>0</v>
       </c>
-      <c r="H64" s="273"/>
+      <c r="H64" s="266"/>
     </row>
     <row r="65" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A65" s="136" t="s">
@@ -5750,7 +5748,7 @@
       <c r="E65" s="162">
         <v>0.94</v>
       </c>
-      <c r="H65" s="273"/>
+      <c r="H65" s="266"/>
     </row>
     <row r="66" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A66" s="136" t="s">
@@ -5768,7 +5766,7 @@
       <c r="E66" s="162">
         <v>0.06</v>
       </c>
-      <c r="H66" s="273"/>
+      <c r="H66" s="266"/>
     </row>
     <row r="67" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A67" s="136" t="s">
@@ -5786,7 +5784,7 @@
       <c r="E67" s="162">
         <v>0</v>
       </c>
-      <c r="H67" s="273"/>
+      <c r="H67" s="266"/>
     </row>
     <row r="68" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A68" s="136" t="s">
@@ -5804,7 +5802,7 @@
       <c r="E68" s="162">
         <v>0.94</v>
       </c>
-      <c r="H68" s="273"/>
+      <c r="H68" s="266"/>
     </row>
     <row r="69" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A69" s="136" t="s">
@@ -5822,7 +5820,7 @@
       <c r="E69" s="162">
         <v>0.06</v>
       </c>
-      <c r="H69" s="273"/>
+      <c r="H69" s="266"/>
     </row>
     <row r="70" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A70" s="136" t="s">
@@ -5840,7 +5838,7 @@
       <c r="E70" s="162">
         <v>0</v>
       </c>
-      <c r="H70" s="273"/>
+      <c r="H70" s="266"/>
     </row>
     <row r="71" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A71" s="136" t="s">
@@ -5858,7 +5856,7 @@
       <c r="E71" s="162">
         <v>0.94</v>
       </c>
-      <c r="H71" s="273"/>
+      <c r="H71" s="266"/>
     </row>
     <row r="72" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A72" s="136" t="s">
@@ -5876,7 +5874,7 @@
       <c r="E72" s="162">
         <v>0.06</v>
       </c>
-      <c r="H72" s="273"/>
+      <c r="H72" s="266"/>
     </row>
     <row r="73" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A73" s="136" t="s">
@@ -5894,7 +5892,7 @@
       <c r="E73" s="162">
         <v>0</v>
       </c>
-      <c r="H73" s="273"/>
+      <c r="H73" s="266"/>
     </row>
     <row r="74" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A74" s="136" t="s">
@@ -5912,7 +5910,7 @@
       <c r="E74" s="162">
         <v>0.94</v>
       </c>
-      <c r="H74" s="273"/>
+      <c r="H74" s="266"/>
     </row>
     <row r="75" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A75" s="136" t="s">
@@ -5930,7 +5928,7 @@
       <c r="E75" s="162">
         <v>0.06</v>
       </c>
-      <c r="H75" s="273"/>
+      <c r="H75" s="266"/>
     </row>
     <row r="76" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A76" s="136" t="s">
@@ -5948,7 +5946,7 @@
       <c r="E76" s="162">
         <v>0</v>
       </c>
-      <c r="H76" s="273"/>
+      <c r="H76" s="266"/>
     </row>
     <row r="77" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A77" s="136" t="s">
@@ -5966,7 +5964,7 @@
       <c r="E77" s="162">
         <v>0.94</v>
       </c>
-      <c r="H77" s="273"/>
+      <c r="H77" s="266"/>
     </row>
     <row r="78" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A78" s="136" t="s">
@@ -5984,7 +5982,7 @@
       <c r="E78" s="162">
         <v>0.06</v>
       </c>
-      <c r="H78" s="273"/>
+      <c r="H78" s="266"/>
     </row>
     <row r="79" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A79" s="136" t="s">
@@ -6002,7 +6000,7 @@
       <c r="E79" s="162">
         <v>0</v>
       </c>
-      <c r="H79" s="273"/>
+      <c r="H79" s="266"/>
     </row>
     <row r="80" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A80" s="136" t="s">
@@ -6020,7 +6018,7 @@
       <c r="E80" s="162">
         <v>0.94</v>
       </c>
-      <c r="H80" s="273"/>
+      <c r="H80" s="266"/>
     </row>
     <row r="81" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A81" s="136" t="s">
@@ -6038,7 +6036,7 @@
       <c r="E81" s="162">
         <v>0.06</v>
       </c>
-      <c r="H81" s="273"/>
+      <c r="H81" s="266"/>
     </row>
     <row r="82" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A82" s="136" t="s">
@@ -6056,7 +6054,7 @@
       <c r="E82" s="162">
         <v>0</v>
       </c>
-      <c r="H82" s="273"/>
+      <c r="H82" s="266"/>
     </row>
     <row r="83" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A83" s="136" t="s">
@@ -6074,7 +6072,7 @@
       <c r="E83" s="162">
         <v>0.94</v>
       </c>
-      <c r="H83" s="273"/>
+      <c r="H83" s="266"/>
     </row>
     <row r="84" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A84" s="136" t="s">
@@ -6092,7 +6090,7 @@
       <c r="E84" s="162">
         <v>0.06</v>
       </c>
-      <c r="H84" s="273"/>
+      <c r="H84" s="266"/>
     </row>
     <row r="85" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A85" s="136" t="s">
@@ -6110,7 +6108,7 @@
       <c r="E85" s="162">
         <v>0</v>
       </c>
-      <c r="H85" s="273"/>
+      <c r="H85" s="266"/>
     </row>
     <row r="86" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A86" s="136" t="s">
@@ -6128,7 +6126,7 @@
       <c r="E86" s="162">
         <v>0.94</v>
       </c>
-      <c r="H86" s="273"/>
+      <c r="H86" s="266"/>
     </row>
     <row r="87" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A87" s="136" t="s">
@@ -6146,7 +6144,7 @@
       <c r="E87" s="162">
         <v>0.06</v>
       </c>
-      <c r="H87" s="273"/>
+      <c r="H87" s="266"/>
     </row>
     <row r="88" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A88" s="136" t="s">
@@ -6164,7 +6162,7 @@
       <c r="E88" s="162">
         <v>0</v>
       </c>
-      <c r="H88" s="273"/>
+      <c r="H88" s="266"/>
     </row>
     <row r="89" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A89" s="136" t="s">
@@ -6182,7 +6180,7 @@
       <c r="E89" s="162">
         <v>0.94</v>
       </c>
-      <c r="H89" s="273"/>
+      <c r="H89" s="266"/>
     </row>
     <row r="90" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A90" s="136" t="s">
@@ -6200,7 +6198,7 @@
       <c r="E90" s="162">
         <v>0.06</v>
       </c>
-      <c r="H90" s="273"/>
+      <c r="H90" s="266"/>
     </row>
     <row r="91" spans="1:8" s="159" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A91" s="136" t="s">
@@ -6219,7 +6217,7 @@
         <v>0</v>
       </c>
       <c r="F91" s="163"/>
-      <c r="H91" s="273"/>
+      <c r="H91" s="266"/>
     </row>
     <row r="92" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A92" s="138" t="s">
@@ -6238,7 +6236,7 @@
         <v>0.96</v>
       </c>
       <c r="F92" s="147"/>
-      <c r="H92" s="274" t="s">
+      <c r="H92" s="267" t="s">
         <v>318</v>
       </c>
     </row>
@@ -6259,7 +6257,7 @@
         <v>0</v>
       </c>
       <c r="F93" s="147"/>
-      <c r="H93" s="274"/>
+      <c r="H93" s="267"/>
     </row>
     <row r="94" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A94" s="138" t="s">
@@ -6278,7 +6276,7 @@
         <v>0.04</v>
       </c>
       <c r="F94" s="147"/>
-      <c r="H94" s="274"/>
+      <c r="H94" s="267"/>
     </row>
     <row r="95" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A95" s="138" t="s">
@@ -6297,7 +6295,7 @@
         <v>0</v>
       </c>
       <c r="F95" s="147"/>
-      <c r="H95" s="274"/>
+      <c r="H95" s="267"/>
     </row>
     <row r="96" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A96" s="138" t="s">
@@ -6316,7 +6314,7 @@
         <v>0.96</v>
       </c>
       <c r="F96" s="147"/>
-      <c r="H96" s="274"/>
+      <c r="H96" s="267"/>
     </row>
     <row r="97" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A97" s="138" t="s">
@@ -6335,7 +6333,7 @@
         <v>0</v>
       </c>
       <c r="F97" s="147"/>
-      <c r="H97" s="274"/>
+      <c r="H97" s="267"/>
     </row>
     <row r="98" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A98" s="138" t="s">
@@ -6354,7 +6352,7 @@
         <v>0.04</v>
       </c>
       <c r="F98" s="147"/>
-      <c r="H98" s="274"/>
+      <c r="H98" s="267"/>
     </row>
     <row r="99" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A99" s="138" t="s">
@@ -6373,7 +6371,7 @@
         <v>0</v>
       </c>
       <c r="F99" s="147"/>
-      <c r="H99" s="274"/>
+      <c r="H99" s="267"/>
     </row>
     <row r="100" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A100" s="138" t="s">
@@ -6392,7 +6390,7 @@
         <v>0.96</v>
       </c>
       <c r="F100" s="147"/>
-      <c r="H100" s="274"/>
+      <c r="H100" s="267"/>
     </row>
     <row r="101" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A101" s="138" t="s">
@@ -6411,7 +6409,7 @@
         <v>0</v>
       </c>
       <c r="F101" s="147"/>
-      <c r="H101" s="274"/>
+      <c r="H101" s="267"/>
     </row>
     <row r="102" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A102" s="138" t="s">
@@ -6430,7 +6428,7 @@
         <v>0.04</v>
       </c>
       <c r="F102" s="147"/>
-      <c r="H102" s="274"/>
+      <c r="H102" s="267"/>
     </row>
     <row r="103" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A103" s="138" t="s">
@@ -6449,7 +6447,7 @@
         <v>0</v>
       </c>
       <c r="F103" s="147"/>
-      <c r="H103" s="274"/>
+      <c r="H103" s="267"/>
     </row>
     <row r="104" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A104" s="138" t="s">
@@ -6468,7 +6466,7 @@
         <v>0.3</v>
       </c>
       <c r="F104" s="147"/>
-      <c r="H104" s="274"/>
+      <c r="H104" s="267"/>
     </row>
     <row r="105" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A105" s="138" t="s">
@@ -6487,7 +6485,7 @@
         <v>0</v>
       </c>
       <c r="F105" s="147"/>
-      <c r="H105" s="274"/>
+      <c r="H105" s="267"/>
     </row>
     <row r="106" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A106" s="138" t="s">
@@ -6506,7 +6504,7 @@
         <v>0.7</v>
       </c>
       <c r="F106" s="147"/>
-      <c r="H106" s="274"/>
+      <c r="H106" s="267"/>
     </row>
     <row r="107" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A107" s="138" t="s">
@@ -6525,7 +6523,7 @@
         <v>0</v>
       </c>
       <c r="F107" s="147"/>
-      <c r="H107" s="274"/>
+      <c r="H107" s="267"/>
     </row>
     <row r="108" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A108" s="138" t="s">
@@ -6544,7 +6542,7 @@
         <v>0</v>
       </c>
       <c r="F108" s="147"/>
-      <c r="H108" s="274"/>
+      <c r="H108" s="267"/>
     </row>
     <row r="109" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A109" s="138" t="s">
@@ -6563,7 +6561,7 @@
         <v>0</v>
       </c>
       <c r="F109" s="147"/>
-      <c r="H109" s="274"/>
+      <c r="H109" s="267"/>
     </row>
     <row r="110" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A110" s="138" t="s">
@@ -6582,7 +6580,7 @@
         <v>1</v>
       </c>
       <c r="F110" s="147"/>
-      <c r="H110" s="274"/>
+      <c r="H110" s="267"/>
     </row>
     <row r="111" spans="1:8" s="148" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A111" s="138" t="s">
@@ -6601,7 +6599,7 @@
         <v>0</v>
       </c>
       <c r="F111" s="147"/>
-      <c r="H111" s="274"/>
+      <c r="H111" s="267"/>
     </row>
     <row r="112" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A112" s="140" t="s">
@@ -6619,7 +6617,7 @@
       <c r="E112" s="166">
         <v>0.7</v>
       </c>
-      <c r="H112" s="275" t="s">
+      <c r="H112" s="268" t="s">
         <v>306</v>
       </c>
     </row>
@@ -6639,7 +6637,7 @@
       <c r="E113" s="166">
         <v>0</v>
       </c>
-      <c r="H113" s="275"/>
+      <c r="H113" s="268"/>
     </row>
     <row r="114" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A114" s="140" t="s">
@@ -6657,7 +6655,7 @@
       <c r="E114" s="166">
         <v>0</v>
       </c>
-      <c r="H114" s="275"/>
+      <c r="H114" s="268"/>
     </row>
     <row r="115" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A115" s="140" t="s">
@@ -6675,7 +6673,7 @@
       <c r="E115" s="166">
         <v>0.3</v>
       </c>
-      <c r="H115" s="275"/>
+      <c r="H115" s="268"/>
     </row>
     <row r="116" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A116" s="140" t="s">
@@ -6693,7 +6691,7 @@
       <c r="E116" s="166">
         <v>0</v>
       </c>
-      <c r="H116" s="275"/>
+      <c r="H116" s="268"/>
     </row>
     <row r="117" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A117" s="140" t="s">
@@ -6711,7 +6709,7 @@
       <c r="E117" s="166">
         <v>0</v>
       </c>
-      <c r="H117" s="275"/>
+      <c r="H117" s="268"/>
     </row>
     <row r="118" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A118" s="140" t="s">
@@ -6729,7 +6727,7 @@
       <c r="E118" s="166">
         <v>0.6</v>
       </c>
-      <c r="H118" s="275"/>
+      <c r="H118" s="268"/>
     </row>
     <row r="119" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A119" s="140" t="s">
@@ -6747,7 +6745,7 @@
       <c r="E119" s="166">
         <v>0</v>
       </c>
-      <c r="H119" s="275"/>
+      <c r="H119" s="268"/>
     </row>
     <row r="120" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A120" s="140" t="s">
@@ -6765,7 +6763,7 @@
       <c r="E120" s="166">
         <v>0</v>
       </c>
-      <c r="H120" s="275"/>
+      <c r="H120" s="268"/>
     </row>
     <row r="121" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A121" s="140" t="s">
@@ -6783,7 +6781,7 @@
       <c r="E121" s="166">
         <v>0.4</v>
       </c>
-      <c r="H121" s="275"/>
+      <c r="H121" s="268"/>
     </row>
     <row r="122" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A122" s="140" t="s">
@@ -6801,7 +6799,7 @@
       <c r="E122" s="166">
         <v>0</v>
       </c>
-      <c r="H122" s="275"/>
+      <c r="H122" s="268"/>
     </row>
     <row r="123" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A123" s="140" t="s">
@@ -6819,7 +6817,7 @@
       <c r="E123" s="166">
         <v>0</v>
       </c>
-      <c r="H123" s="275"/>
+      <c r="H123" s="268"/>
     </row>
     <row r="124" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A124" s="140" t="s">
@@ -6837,7 +6835,7 @@
       <c r="E124" s="166">
         <v>0.42</v>
       </c>
-      <c r="H124" s="275"/>
+      <c r="H124" s="268"/>
     </row>
     <row r="125" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A125" s="140" t="s">
@@ -6855,7 +6853,7 @@
       <c r="E125" s="166">
         <v>0</v>
       </c>
-      <c r="H125" s="275"/>
+      <c r="H125" s="268"/>
     </row>
     <row r="126" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A126" s="140" t="s">
@@ -6873,7 +6871,7 @@
       <c r="E126" s="166">
         <v>0</v>
       </c>
-      <c r="H126" s="275"/>
+      <c r="H126" s="268"/>
     </row>
     <row r="127" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A127" s="140" t="s">
@@ -6891,7 +6889,7 @@
       <c r="E127" s="166">
         <v>0.57999999999999996</v>
       </c>
-      <c r="H127" s="275"/>
+      <c r="H127" s="268"/>
     </row>
     <row r="128" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A128" s="140" t="s">
@@ -6909,7 +6907,7 @@
       <c r="E128" s="166">
         <v>0</v>
       </c>
-      <c r="H128" s="275"/>
+      <c r="H128" s="268"/>
     </row>
     <row r="129" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A129" s="140" t="s">
@@ -6927,7 +6925,7 @@
       <c r="E129" s="166">
         <v>0</v>
       </c>
-      <c r="H129" s="275"/>
+      <c r="H129" s="268"/>
     </row>
     <row r="130" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A130" s="140" t="s">
@@ -6945,7 +6943,7 @@
       <c r="E130" s="166">
         <v>0.05</v>
       </c>
-      <c r="H130" s="275"/>
+      <c r="H130" s="268"/>
     </row>
     <row r="131" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A131" s="140" t="s">
@@ -6963,7 +6961,7 @@
       <c r="E131" s="166">
         <v>0</v>
       </c>
-      <c r="H131" s="275"/>
+      <c r="H131" s="268"/>
     </row>
     <row r="132" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A132" s="140" t="s">
@@ -6981,7 +6979,7 @@
       <c r="E132" s="166">
         <v>0</v>
       </c>
-      <c r="H132" s="275"/>
+      <c r="H132" s="268"/>
     </row>
     <row r="133" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A133" s="140" t="s">
@@ -6999,7 +6997,7 @@
       <c r="E133" s="166">
         <v>0.95</v>
       </c>
-      <c r="H133" s="275"/>
+      <c r="H133" s="268"/>
     </row>
     <row r="134" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A134" s="140" t="s">
@@ -7017,7 +7015,7 @@
       <c r="E134" s="166">
         <v>0</v>
       </c>
-      <c r="H134" s="275"/>
+      <c r="H134" s="268"/>
     </row>
     <row r="135" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A135" s="140" t="s">
@@ -7035,7 +7033,7 @@
       <c r="E135" s="166">
         <v>0</v>
       </c>
-      <c r="H135" s="275"/>
+      <c r="H135" s="268"/>
     </row>
     <row r="136" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A136" s="140" t="s">
@@ -7053,7 +7051,7 @@
       <c r="E136" s="166">
         <v>0</v>
       </c>
-      <c r="H136" s="275"/>
+      <c r="H136" s="268"/>
     </row>
     <row r="137" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A137" s="140" t="s">
@@ -7071,7 +7069,7 @@
       <c r="E137" s="166">
         <v>0</v>
       </c>
-      <c r="H137" s="275"/>
+      <c r="H137" s="268"/>
     </row>
     <row r="138" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A138" s="140" t="s">
@@ -7089,7 +7087,7 @@
       <c r="E138" s="166">
         <v>0</v>
       </c>
-      <c r="H138" s="275"/>
+      <c r="H138" s="268"/>
     </row>
     <row r="139" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A139" s="140" t="s">
@@ -7107,7 +7105,7 @@
       <c r="E139" s="166">
         <v>0.05</v>
       </c>
-      <c r="H139" s="275"/>
+      <c r="H139" s="268"/>
     </row>
     <row r="140" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A140" s="140" t="s">
@@ -7125,7 +7123,7 @@
       <c r="E140" s="166">
         <v>0.95</v>
       </c>
-      <c r="H140" s="275"/>
+      <c r="H140" s="268"/>
     </row>
     <row r="141" spans="1:8" s="167" customFormat="1" x14ac:dyDescent="0.2">
       <c r="A141" s="140" t="s">
@@ -7143,7 +7141,7 @@
       <c r="E141" s="166">
         <v>0</v>
       </c>
-      <c r="H141" s="275"/>
+      <c r="H141" s="268"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -7189,7 +7187,7 @@
         <v>0.96499999999999997</v>
       </c>
       <c r="D2" s="64"/>
-      <c r="E2" s="276" t="s">
+      <c r="E2" s="269" t="s">
         <v>317</v>
       </c>
     </row>
@@ -7204,7 +7202,7 @@
         <v>0.96499999999999997</v>
       </c>
       <c r="D3" s="64"/>
-      <c r="E3" s="276"/>
+      <c r="E3" s="269"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A4" s="136" t="s">
@@ -7217,7 +7215,7 @@
         <v>0.5</v>
       </c>
       <c r="D4" s="64"/>
-      <c r="E4" s="276"/>
+      <c r="E4" s="269"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A5" s="136" t="s">
@@ -7230,7 +7228,7 @@
         <v>0</v>
       </c>
       <c r="D5" s="64"/>
-      <c r="E5" s="276"/>
+      <c r="E5" s="269"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A6" s="138" t="s">
@@ -7243,7 +7241,7 @@
         <v>0.96499999999999997</v>
       </c>
       <c r="D6" s="64"/>
-      <c r="E6" s="276"/>
+      <c r="E6" s="269"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A7" s="138" t="s">
@@ -7256,7 +7254,7 @@
         <v>0.96499999999999997</v>
       </c>
       <c r="D7" s="64"/>
-      <c r="E7" s="276"/>
+      <c r="E7" s="269"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A8" s="138" t="s">
@@ -7269,7 +7267,7 @@
         <v>0.5</v>
       </c>
       <c r="D8" s="64"/>
-      <c r="E8" s="276"/>
+      <c r="E8" s="269"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A9" s="138" t="s">
@@ -7282,7 +7280,7 @@
         <v>0</v>
       </c>
       <c r="D9" s="64"/>
-      <c r="E9" s="276"/>
+      <c r="E9" s="269"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A10" s="140" t="s">
@@ -7295,7 +7293,7 @@
         <v>0.96499999999999997</v>
       </c>
       <c r="D10" s="64"/>
-      <c r="E10" s="276"/>
+      <c r="E10" s="269"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="140" t="s">
@@ -7308,7 +7306,7 @@
         <v>0.96499999999999997</v>
       </c>
       <c r="D11" s="64"/>
-      <c r="E11" s="276"/>
+      <c r="E11" s="269"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="140" t="s">
@@ -7321,7 +7319,7 @@
         <v>0.96499999999999997</v>
       </c>
       <c r="D12" s="64"/>
-      <c r="E12" s="276"/>
+      <c r="E12" s="269"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A13" s="140" t="s">
@@ -7334,7 +7332,7 @@
         <v>0</v>
       </c>
       <c r="D13" s="64"/>
-      <c r="E13" s="276"/>
+      <c r="E13" s="269"/>
     </row>
     <row r="18" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B18" s="64"/>
@@ -7467,84 +7465,84 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:21" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="293" t="s">
+      <c r="B2" s="287" t="s">
         <v>152</v>
       </c>
-      <c r="C2" s="295" t="s">
+      <c r="C2" s="273" t="s">
         <v>8</v>
       </c>
-      <c r="D2" s="296"/>
-      <c r="E2" s="296"/>
-      <c r="F2" s="297"/>
-      <c r="G2" s="310" t="s">
+      <c r="D2" s="274"/>
+      <c r="E2" s="274"/>
+      <c r="F2" s="289"/>
+      <c r="G2" s="285" t="s">
         <v>9</v>
       </c>
-      <c r="H2" s="293" t="s">
+      <c r="H2" s="287" t="s">
         <v>263</v>
       </c>
-      <c r="I2" s="295" t="s">
+      <c r="I2" s="273" t="s">
         <v>10</v>
       </c>
-      <c r="J2" s="296"/>
-      <c r="K2" s="305"/>
+      <c r="J2" s="274"/>
+      <c r="K2" s="275"/>
     </row>
     <row r="3" spans="1:21" ht="17" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B3" s="294"/>
-      <c r="C3" s="298"/>
-      <c r="D3" s="299"/>
-      <c r="E3" s="299"/>
-      <c r="F3" s="300"/>
-      <c r="G3" s="311"/>
-      <c r="H3" s="294"/>
-      <c r="I3" s="298"/>
-      <c r="J3" s="299"/>
-      <c r="K3" s="306"/>
+      <c r="B3" s="288"/>
+      <c r="C3" s="276"/>
+      <c r="D3" s="277"/>
+      <c r="E3" s="277"/>
+      <c r="F3" s="290"/>
+      <c r="G3" s="286"/>
+      <c r="H3" s="288"/>
+      <c r="I3" s="276"/>
+      <c r="J3" s="277"/>
+      <c r="K3" s="278"/>
     </row>
     <row r="4" spans="1:21" s="44" customFormat="1" ht="270" x14ac:dyDescent="0.2">
       <c r="A4" s="46"/>
       <c r="B4" s="174" t="s">
         <v>153</v>
       </c>
-      <c r="C4" s="301" t="s">
+      <c r="C4" s="291" t="s">
         <v>321</v>
       </c>
-      <c r="D4" s="302"/>
-      <c r="E4" s="302"/>
-      <c r="F4" s="303"/>
+      <c r="D4" s="292"/>
+      <c r="E4" s="292"/>
+      <c r="F4" s="293"/>
       <c r="G4" s="175" t="s">
         <v>270</v>
       </c>
       <c r="H4" s="176" t="s">
         <v>271</v>
       </c>
-      <c r="I4" s="307" t="s">
+      <c r="I4" s="282" t="s">
         <v>295</v>
       </c>
-      <c r="J4" s="308"/>
-      <c r="K4" s="309"/>
+      <c r="J4" s="283"/>
+      <c r="K4" s="284"/>
     </row>
     <row r="5" spans="1:21" s="44" customFormat="1" ht="37" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A5" s="46"/>
       <c r="B5" s="92" t="s">
         <v>154</v>
       </c>
-      <c r="C5" s="277" t="s">
+      <c r="C5" s="279" t="s">
         <v>322</v>
       </c>
-      <c r="D5" s="278"/>
-      <c r="E5" s="278"/>
-      <c r="F5" s="304"/>
+      <c r="D5" s="280"/>
+      <c r="E5" s="280"/>
+      <c r="F5" s="281"/>
       <c r="G5" s="177">
         <v>0.8</v>
       </c>
       <c r="H5" s="178" t="s">
         <v>307</v>
       </c>
-      <c r="I5" s="280" t="s">
+      <c r="I5" s="270" t="s">
         <v>269</v>
       </c>
-      <c r="J5" s="281"/>
-      <c r="K5" s="282"/>
+      <c r="J5" s="271"/>
+      <c r="K5" s="272"/>
       <c r="L5" s="5"/>
       <c r="M5" s="5"/>
       <c r="N5" s="5"/>
@@ -7554,23 +7552,23 @@
       <c r="B6" s="92" t="s">
         <v>155</v>
       </c>
-      <c r="C6" s="277" t="s">
+      <c r="C6" s="279" t="s">
         <v>323</v>
       </c>
-      <c r="D6" s="278"/>
-      <c r="E6" s="278"/>
-      <c r="F6" s="304"/>
+      <c r="D6" s="280"/>
+      <c r="E6" s="280"/>
+      <c r="F6" s="281"/>
       <c r="G6" s="177">
         <v>0.8</v>
       </c>
       <c r="H6" s="179" t="s">
         <v>307</v>
       </c>
-      <c r="I6" s="280" t="s">
+      <c r="I6" s="270" t="s">
         <v>268</v>
       </c>
-      <c r="J6" s="281"/>
-      <c r="K6" s="282"/>
+      <c r="J6" s="271"/>
+      <c r="K6" s="272"/>
       <c r="L6" s="5"/>
       <c r="M6" s="5"/>
       <c r="N6" s="5"/>
@@ -7580,21 +7578,21 @@
       <c r="B7" s="92" t="s">
         <v>297</v>
       </c>
-      <c r="C7" s="277" t="s">
+      <c r="C7" s="279" t="s">
         <v>298</v>
       </c>
-      <c r="D7" s="278"/>
-      <c r="E7" s="278"/>
-      <c r="F7" s="304"/>
+      <c r="D7" s="280"/>
+      <c r="E7" s="280"/>
+      <c r="F7" s="281"/>
       <c r="G7" s="177">
         <v>1</v>
       </c>
       <c r="H7" s="179"/>
-      <c r="I7" s="280" t="s">
+      <c r="I7" s="270" t="s">
         <v>299</v>
       </c>
-      <c r="J7" s="281"/>
-      <c r="K7" s="282"/>
+      <c r="J7" s="271"/>
+      <c r="K7" s="272"/>
       <c r="L7" s="5"/>
       <c r="M7" s="5"/>
       <c r="N7" s="5"/>
@@ -7604,21 +7602,21 @@
       <c r="B8" s="92" t="s">
         <v>156</v>
       </c>
-      <c r="C8" s="277" t="s">
+      <c r="C8" s="279" t="s">
         <v>265</v>
       </c>
-      <c r="D8" s="278"/>
-      <c r="E8" s="278"/>
-      <c r="F8" s="304"/>
+      <c r="D8" s="280"/>
+      <c r="E8" s="280"/>
+      <c r="F8" s="281"/>
       <c r="G8" s="177">
         <v>1</v>
       </c>
       <c r="H8" s="178" t="s">
         <v>266</v>
       </c>
-      <c r="I8" s="280"/>
-      <c r="J8" s="281"/>
-      <c r="K8" s="282"/>
+      <c r="I8" s="270"/>
+      <c r="J8" s="271"/>
+      <c r="K8" s="272"/>
       <c r="L8" s="5"/>
       <c r="M8" s="5"/>
       <c r="N8" s="5"/>
@@ -7628,23 +7626,23 @@
       <c r="B9" s="92" t="s">
         <v>157</v>
       </c>
-      <c r="C9" s="277" t="s">
+      <c r="C9" s="279" t="s">
         <v>158</v>
       </c>
-      <c r="D9" s="278"/>
-      <c r="E9" s="278"/>
-      <c r="F9" s="304"/>
+      <c r="D9" s="280"/>
+      <c r="E9" s="280"/>
+      <c r="F9" s="281"/>
       <c r="G9" s="177">
         <v>0.95</v>
       </c>
       <c r="H9" s="178" t="s">
         <v>307</v>
       </c>
-      <c r="I9" s="277" t="s">
+      <c r="I9" s="279" t="s">
         <v>264</v>
       </c>
-      <c r="J9" s="278"/>
-      <c r="K9" s="279"/>
+      <c r="J9" s="280"/>
+      <c r="K9" s="296"/>
       <c r="L9" s="5"/>
       <c r="M9" s="5"/>
       <c r="N9" s="5"/>
@@ -7654,21 +7652,21 @@
       <c r="B10" s="92" t="s">
         <v>159</v>
       </c>
-      <c r="C10" s="277" t="s">
+      <c r="C10" s="279" t="s">
         <v>162</v>
       </c>
-      <c r="D10" s="278"/>
-      <c r="E10" s="278"/>
-      <c r="F10" s="304"/>
+      <c r="D10" s="280"/>
+      <c r="E10" s="280"/>
+      <c r="F10" s="281"/>
       <c r="G10" s="180">
         <v>0.9</v>
       </c>
       <c r="H10" s="178"/>
-      <c r="I10" s="280" t="s">
+      <c r="I10" s="270" t="s">
         <v>267</v>
       </c>
-      <c r="J10" s="281"/>
-      <c r="K10" s="282"/>
+      <c r="J10" s="271"/>
+      <c r="K10" s="272"/>
       <c r="L10" s="5"/>
       <c r="M10" s="5"/>
       <c r="N10" s="5"/>
@@ -7678,21 +7676,21 @@
       <c r="B11" s="92" t="s">
         <v>160</v>
       </c>
-      <c r="C11" s="277" t="s">
+      <c r="C11" s="279" t="s">
         <v>161</v>
       </c>
-      <c r="D11" s="278"/>
-      <c r="E11" s="278"/>
-      <c r="F11" s="304"/>
+      <c r="D11" s="280"/>
+      <c r="E11" s="280"/>
+      <c r="F11" s="281"/>
       <c r="G11" s="180">
         <v>0.9</v>
       </c>
       <c r="H11" s="179"/>
-      <c r="I11" s="280" t="s">
+      <c r="I11" s="270" t="s">
         <v>267</v>
       </c>
-      <c r="J11" s="281"/>
-      <c r="K11" s="282"/>
+      <c r="J11" s="271"/>
+      <c r="K11" s="272"/>
       <c r="L11" s="5"/>
       <c r="M11" s="5"/>
       <c r="N11" s="5"/>
@@ -7723,28 +7721,28 @@
       <c r="U13" s="51"/>
     </row>
     <row r="14" spans="1:21" ht="30" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B14" s="287" t="s">
+      <c r="B14" s="301" t="s">
         <v>258</v>
       </c>
-      <c r="C14" s="288"/>
-      <c r="D14" s="288"/>
-      <c r="E14" s="288"/>
-      <c r="F14" s="288"/>
-      <c r="G14" s="288"/>
-      <c r="H14" s="288"/>
-      <c r="I14" s="288"/>
-      <c r="J14" s="288"/>
-      <c r="K14" s="288"/>
-      <c r="L14" s="288"/>
-      <c r="M14" s="288"/>
-      <c r="N14" s="288"/>
-      <c r="O14" s="288"/>
-      <c r="P14" s="288"/>
-      <c r="Q14" s="288"/>
-      <c r="R14" s="288"/>
-      <c r="S14" s="288"/>
-      <c r="T14" s="288"/>
-      <c r="U14" s="289"/>
+      <c r="C14" s="302"/>
+      <c r="D14" s="302"/>
+      <c r="E14" s="302"/>
+      <c r="F14" s="302"/>
+      <c r="G14" s="302"/>
+      <c r="H14" s="302"/>
+      <c r="I14" s="302"/>
+      <c r="J14" s="302"/>
+      <c r="K14" s="302"/>
+      <c r="L14" s="302"/>
+      <c r="M14" s="302"/>
+      <c r="N14" s="302"/>
+      <c r="O14" s="302"/>
+      <c r="P14" s="302"/>
+      <c r="Q14" s="302"/>
+      <c r="R14" s="302"/>
+      <c r="S14" s="302"/>
+      <c r="T14" s="302"/>
+      <c r="U14" s="303"/>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.2">
       <c r="B15" s="52"/>
@@ -7769,34 +7767,34 @@
       <c r="U15" s="55"/>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.2">
-      <c r="B16" s="285" t="s">
+      <c r="B16" s="299" t="s">
         <v>254</v>
       </c>
-      <c r="C16" s="286"/>
-      <c r="D16" s="286"/>
-      <c r="E16" s="286"/>
-      <c r="F16" s="286"/>
-      <c r="G16" s="286"/>
-      <c r="H16" s="286"/>
-      <c r="I16" s="286"/>
-      <c r="J16" s="286"/>
-      <c r="K16" s="286"/>
-      <c r="L16" s="286"/>
-      <c r="M16" s="286"/>
-      <c r="N16" s="286"/>
-      <c r="O16" s="286"/>
-      <c r="P16" s="286"/>
-      <c r="Q16" s="286"/>
-      <c r="R16" s="286"/>
-      <c r="S16" s="286"/>
-      <c r="T16" s="286"/>
-      <c r="U16" s="292"/>
+      <c r="C16" s="300"/>
+      <c r="D16" s="300"/>
+      <c r="E16" s="300"/>
+      <c r="F16" s="300"/>
+      <c r="G16" s="300"/>
+      <c r="H16" s="300"/>
+      <c r="I16" s="300"/>
+      <c r="J16" s="300"/>
+      <c r="K16" s="300"/>
+      <c r="L16" s="300"/>
+      <c r="M16" s="300"/>
+      <c r="N16" s="300"/>
+      <c r="O16" s="300"/>
+      <c r="P16" s="300"/>
+      <c r="Q16" s="300"/>
+      <c r="R16" s="300"/>
+      <c r="S16" s="300"/>
+      <c r="T16" s="300"/>
+      <c r="U16" s="304"/>
     </row>
     <row r="17" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B17" s="290" t="s">
+      <c r="B17" s="294" t="s">
         <v>250</v>
       </c>
-      <c r="C17" s="291"/>
+      <c r="C17" s="295"/>
       <c r="D17" s="181">
         <v>2008</v>
       </c>
@@ -7853,10 +7851,10 @@
       </c>
     </row>
     <row r="18" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B18" s="290" t="s">
+      <c r="B18" s="294" t="s">
         <v>251</v>
       </c>
-      <c r="C18" s="291"/>
+      <c r="C18" s="295"/>
       <c r="D18" s="59">
         <v>0.86</v>
       </c>
@@ -7913,10 +7911,10 @@
       </c>
     </row>
     <row r="19" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B19" s="290" t="s">
+      <c r="B19" s="294" t="s">
         <v>252</v>
       </c>
-      <c r="C19" s="291"/>
+      <c r="C19" s="295"/>
       <c r="D19" s="59">
         <f>78/86</f>
         <v>0.90697674418604646</v>
@@ -7988,10 +7986,10 @@
       </c>
     </row>
     <row r="20" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B20" s="290" t="s">
+      <c r="B20" s="294" t="s">
         <v>253</v>
       </c>
-      <c r="C20" s="291"/>
+      <c r="C20" s="295"/>
       <c r="D20" s="59">
         <v>1</v>
       </c>
@@ -8070,17 +8068,17 @@
       <c r="U21" s="55"/>
     </row>
     <row r="22" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B22" s="285" t="s">
+      <c r="B22" s="299" t="s">
         <v>257</v>
       </c>
-      <c r="C22" s="286"/>
-      <c r="D22" s="286"/>
-      <c r="E22" s="286"/>
-      <c r="F22" s="286"/>
-      <c r="G22" s="286"/>
-      <c r="H22" s="286"/>
-      <c r="I22" s="286"/>
-      <c r="J22" s="286"/>
+      <c r="C22" s="300"/>
+      <c r="D22" s="300"/>
+      <c r="E22" s="300"/>
+      <c r="F22" s="300"/>
+      <c r="G22" s="300"/>
+      <c r="H22" s="300"/>
+      <c r="I22" s="300"/>
+      <c r="J22" s="300"/>
       <c r="K22" s="184"/>
       <c r="L22" s="184"/>
       <c r="M22" s="184"/>
@@ -8094,10 +8092,10 @@
       <c r="U22" s="185"/>
     </row>
     <row r="23" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B23" s="290" t="s">
+      <c r="B23" s="294" t="s">
         <v>250</v>
       </c>
-      <c r="C23" s="291"/>
+      <c r="C23" s="295"/>
       <c r="D23" s="181">
         <v>2019</v>
       </c>
@@ -8132,10 +8130,10 @@
       <c r="U23" s="55"/>
     </row>
     <row r="24" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B24" s="290" t="s">
+      <c r="B24" s="294" t="s">
         <v>251</v>
       </c>
-      <c r="C24" s="291"/>
+      <c r="C24" s="295"/>
       <c r="D24" s="59">
         <f>E24</f>
         <v>0.53</v>
@@ -8173,10 +8171,10 @@
       <c r="U24" s="55"/>
     </row>
     <row r="25" spans="2:21" x14ac:dyDescent="0.2">
-      <c r="B25" s="290" t="s">
+      <c r="B25" s="294" t="s">
         <v>252</v>
       </c>
-      <c r="C25" s="291"/>
+      <c r="C25" s="295"/>
       <c r="D25" s="59">
         <f>E25</f>
         <v>0.35830985915492958</v>
@@ -8214,10 +8212,10 @@
       <c r="U25" s="55"/>
     </row>
     <row r="26" spans="2:21" ht="15" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B26" s="283" t="s">
+      <c r="B26" s="297" t="s">
         <v>253</v>
       </c>
-      <c r="C26" s="284"/>
+      <c r="C26" s="298"/>
       <c r="D26" s="186">
         <v>0</v>
       </c>
@@ -8282,26 +8280,6 @@
     </row>
   </sheetData>
   <mergeCells count="32">
-    <mergeCell ref="I8:K8"/>
-    <mergeCell ref="I2:K3"/>
-    <mergeCell ref="C7:F7"/>
-    <mergeCell ref="I7:K7"/>
-    <mergeCell ref="I4:K4"/>
-    <mergeCell ref="C5:F5"/>
-    <mergeCell ref="C6:F6"/>
-    <mergeCell ref="G2:G3"/>
-    <mergeCell ref="H2:H3"/>
-    <mergeCell ref="I5:K5"/>
-    <mergeCell ref="I6:K6"/>
-    <mergeCell ref="B2:B3"/>
-    <mergeCell ref="C2:F3"/>
-    <mergeCell ref="C4:F4"/>
-    <mergeCell ref="B24:C24"/>
-    <mergeCell ref="B25:C25"/>
-    <mergeCell ref="C11:F11"/>
-    <mergeCell ref="C8:F8"/>
-    <mergeCell ref="C9:F9"/>
-    <mergeCell ref="C10:F10"/>
     <mergeCell ref="I9:K9"/>
     <mergeCell ref="I10:K10"/>
     <mergeCell ref="B26:C26"/>
@@ -8314,6 +8292,26 @@
     <mergeCell ref="B23:C23"/>
     <mergeCell ref="B16:U16"/>
     <mergeCell ref="I11:K11"/>
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:F3"/>
+    <mergeCell ref="C4:F4"/>
+    <mergeCell ref="B24:C24"/>
+    <mergeCell ref="B25:C25"/>
+    <mergeCell ref="C11:F11"/>
+    <mergeCell ref="C8:F8"/>
+    <mergeCell ref="C9:F9"/>
+    <mergeCell ref="C10:F10"/>
+    <mergeCell ref="I8:K8"/>
+    <mergeCell ref="I2:K3"/>
+    <mergeCell ref="C7:F7"/>
+    <mergeCell ref="I7:K7"/>
+    <mergeCell ref="I4:K4"/>
+    <mergeCell ref="C5:F5"/>
+    <mergeCell ref="C6:F6"/>
+    <mergeCell ref="G2:G3"/>
+    <mergeCell ref="H2:H3"/>
+    <mergeCell ref="I5:K5"/>
+    <mergeCell ref="I6:K6"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" fitToWidth="0" fitToHeight="0" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
@@ -8359,13 +8357,13 @@
       </c>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B3" s="211" t="s">
+      <c r="B3" s="210" t="s">
         <v>243</v>
       </c>
-      <c r="C3" s="212"/>
-      <c r="D3" s="212"/>
-      <c r="E3" s="212"/>
-      <c r="F3" s="213"/>
+      <c r="C3" s="211"/>
+      <c r="D3" s="211"/>
+      <c r="E3" s="211"/>
+      <c r="F3" s="212"/>
       <c r="G3" s="75"/>
       <c r="H3" s="76"/>
     </row>
@@ -8392,237 +8390,237 @@
       </c>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B5" s="211" t="s">
+      <c r="B5" s="210" t="s">
         <v>260</v>
       </c>
-      <c r="C5" s="212"/>
-      <c r="D5" s="212"/>
-      <c r="E5" s="212"/>
-      <c r="F5" s="213"/>
+      <c r="C5" s="211"/>
+      <c r="D5" s="211"/>
+      <c r="E5" s="211"/>
+      <c r="F5" s="212"/>
       <c r="G5" s="65"/>
       <c r="H5" s="194"/>
     </row>
-    <row r="6" spans="2:8" s="317" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="312" t="s">
+    <row r="6" spans="2:8" x14ac:dyDescent="0.2">
+      <c r="B6" s="207" t="s">
         <v>164</v>
       </c>
-      <c r="C6" s="313" t="s">
+      <c r="C6" s="64" t="s">
         <v>261</v>
       </c>
-      <c r="D6" s="313">
+      <c r="D6" s="64">
         <v>0.8</v>
       </c>
-      <c r="E6" s="314" t="s">
+      <c r="E6" s="208" t="s">
         <v>262</v>
       </c>
-      <c r="F6" s="315" t="s">
+      <c r="F6" s="209" t="s">
         <v>272</v>
       </c>
-      <c r="G6" s="314">
+      <c r="G6" s="208">
         <v>3</v>
       </c>
-      <c r="H6" s="316">
+      <c r="H6" s="194">
         <f>H4*G6</f>
         <v>6</v>
       </c>
     </row>
     <row r="7" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B7" s="211" t="s">
+      <c r="B7" s="210" t="s">
         <v>273</v>
       </c>
-      <c r="C7" s="212"/>
-      <c r="D7" s="212"/>
-      <c r="E7" s="212"/>
-      <c r="F7" s="213"/>
+      <c r="C7" s="211"/>
+      <c r="D7" s="211"/>
+      <c r="E7" s="211"/>
+      <c r="F7" s="212"/>
       <c r="G7" s="65"/>
       <c r="H7" s="194"/>
     </row>
-    <row r="8" spans="2:8" s="201" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="204" t="s">
+    <row r="8" spans="2:8" s="202" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="313" t="s">
         <v>164</v>
       </c>
-      <c r="C8" s="205" t="s">
+      <c r="C8" s="314" t="s">
         <v>290</v>
       </c>
-      <c r="D8" s="198">
+      <c r="D8" s="315">
         <v>0.68</v>
       </c>
-      <c r="E8" s="198" t="s">
+      <c r="E8" s="315" t="s">
         <v>292</v>
       </c>
       <c r="F8" s="217" t="s">
         <v>294</v>
       </c>
-      <c r="G8" s="226">
+      <c r="G8" s="215">
         <v>3</v>
       </c>
-      <c r="H8" s="218">
+      <c r="H8" s="216">
         <f>H6*G8</f>
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="2:8" s="201" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="204" t="s">
+    <row r="9" spans="2:8" s="202" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="313" t="s">
         <v>164</v>
       </c>
-      <c r="C9" s="205" t="s">
+      <c r="C9" s="314" t="s">
         <v>291</v>
       </c>
-      <c r="D9" s="198">
+      <c r="D9" s="315">
         <v>0.76</v>
       </c>
-      <c r="E9" s="198" t="s">
+      <c r="E9" s="315" t="s">
         <v>293</v>
       </c>
       <c r="F9" s="217"/>
-      <c r="G9" s="226"/>
-      <c r="H9" s="218"/>
-    </row>
-    <row r="10" spans="2:8" s="201" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="196" t="s">
+      <c r="G9" s="215"/>
+      <c r="H9" s="216"/>
+    </row>
+    <row r="10" spans="2:8" s="202" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="203" t="s">
         <v>164</v>
       </c>
-      <c r="C10" s="205" t="s">
+      <c r="C10" s="314" t="s">
         <v>154</v>
       </c>
-      <c r="D10" s="197">
+      <c r="D10" s="167">
         <v>0.8</v>
       </c>
-      <c r="E10" s="198" t="s">
+      <c r="E10" s="315" t="s">
         <v>274</v>
       </c>
       <c r="F10" s="217"/>
-      <c r="G10" s="226"/>
-      <c r="H10" s="218"/>
-    </row>
-    <row r="11" spans="2:8" s="201" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B11" s="196" t="s">
+      <c r="G10" s="215"/>
+      <c r="H10" s="216"/>
+    </row>
+    <row r="11" spans="2:8" s="202" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="203" t="s">
         <v>164</v>
       </c>
-      <c r="C11" s="197" t="s">
+      <c r="C11" s="167" t="s">
         <v>155</v>
       </c>
-      <c r="D11" s="197">
+      <c r="D11" s="167">
         <v>0.8</v>
       </c>
-      <c r="E11" s="198" t="s">
+      <c r="E11" s="315" t="s">
         <v>274</v>
       </c>
       <c r="F11" s="217"/>
-      <c r="G11" s="226"/>
-      <c r="H11" s="218"/>
-    </row>
-    <row r="12" spans="2:8" s="201" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="196" t="s">
+      <c r="G11" s="215"/>
+      <c r="H11" s="216"/>
+    </row>
+    <row r="12" spans="2:8" s="202" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="203" t="s">
         <v>164</v>
       </c>
-      <c r="C12" s="197" t="s">
+      <c r="C12" s="167" t="s">
         <v>159</v>
       </c>
-      <c r="D12" s="197">
+      <c r="D12" s="167">
         <v>0.9</v>
       </c>
-      <c r="E12" s="198" t="s">
+      <c r="E12" s="315" t="s">
         <v>280</v>
       </c>
       <c r="F12" s="217"/>
-      <c r="G12" s="226"/>
-      <c r="H12" s="218"/>
-    </row>
-    <row r="13" spans="2:8" s="201" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B13" s="196" t="s">
+      <c r="G12" s="215"/>
+      <c r="H12" s="216"/>
+    </row>
+    <row r="13" spans="2:8" s="202" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B13" s="203" t="s">
         <v>164</v>
       </c>
-      <c r="C13" s="197" t="s">
+      <c r="C13" s="167" t="s">
         <v>160</v>
       </c>
-      <c r="D13" s="197">
+      <c r="D13" s="167">
         <v>0.9</v>
       </c>
-      <c r="E13" s="198" t="s">
+      <c r="E13" s="315" t="s">
         <v>275</v>
       </c>
       <c r="F13" s="217"/>
-      <c r="G13" s="226"/>
-      <c r="H13" s="218"/>
+      <c r="G13" s="215"/>
+      <c r="H13" s="216"/>
     </row>
     <row r="14" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B14" s="211" t="s">
+      <c r="B14" s="210" t="s">
         <v>305</v>
       </c>
-      <c r="C14" s="212"/>
-      <c r="D14" s="212"/>
-      <c r="E14" s="212"/>
-      <c r="F14" s="213"/>
+      <c r="C14" s="211"/>
+      <c r="D14" s="211"/>
+      <c r="E14" s="211"/>
+      <c r="F14" s="212"/>
       <c r="G14" s="65"/>
       <c r="H14" s="194"/>
     </row>
-    <row r="15" spans="2:8" s="202" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="203" t="s">
+    <row r="15" spans="2:8" s="201" customFormat="1" ht="16" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="196" t="s">
         <v>149</v>
       </c>
-      <c r="C15" s="167" t="s">
+      <c r="C15" s="197" t="s">
         <v>276</v>
       </c>
-      <c r="D15" s="167">
-        <v>0</v>
-      </c>
-      <c r="E15" s="167">
+      <c r="D15" s="197">
+        <v>0</v>
+      </c>
+      <c r="E15" s="197">
         <v>0.1</v>
       </c>
-      <c r="F15" s="214" t="s">
+      <c r="F15" s="218" t="s">
         <v>279</v>
       </c>
-      <c r="G15" s="215">
+      <c r="G15" s="311">
         <v>2</v>
       </c>
-      <c r="H15" s="216">
+      <c r="H15" s="312">
         <f>H8*G15</f>
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="2:8" s="202" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B16" s="203" t="s">
+    <row r="16" spans="2:8" s="201" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B16" s="196" t="s">
         <v>149</v>
       </c>
-      <c r="C16" s="167" t="s">
+      <c r="C16" s="197" t="s">
         <v>277</v>
       </c>
-      <c r="D16" s="167">
-        <v>0</v>
-      </c>
-      <c r="E16" s="167">
+      <c r="D16" s="197">
+        <v>0</v>
+      </c>
+      <c r="E16" s="197">
         <v>0.1</v>
       </c>
-      <c r="F16" s="214"/>
-      <c r="G16" s="215"/>
-      <c r="H16" s="216"/>
-    </row>
-    <row r="17" spans="2:8" s="202" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B17" s="203" t="s">
+      <c r="F16" s="218"/>
+      <c r="G16" s="311"/>
+      <c r="H16" s="312"/>
+    </row>
+    <row r="17" spans="2:8" s="201" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B17" s="196" t="s">
         <v>149</v>
       </c>
-      <c r="C17" s="167" t="s">
+      <c r="C17" s="197" t="s">
         <v>278</v>
       </c>
-      <c r="D17" s="167">
-        <v>0</v>
-      </c>
-      <c r="E17" s="167">
+      <c r="D17" s="197">
+        <v>0</v>
+      </c>
+      <c r="E17" s="197">
         <v>0.1</v>
       </c>
-      <c r="F17" s="214"/>
-      <c r="G17" s="215"/>
-      <c r="H17" s="216"/>
+      <c r="F17" s="218"/>
+      <c r="G17" s="311"/>
+      <c r="H17" s="312"/>
     </row>
     <row r="18" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B18" s="211" t="s">
+      <c r="B18" s="210" t="s">
         <v>324</v>
       </c>
-      <c r="C18" s="212"/>
-      <c r="D18" s="212"/>
-      <c r="E18" s="212"/>
-      <c r="F18" s="213"/>
+      <c r="C18" s="211"/>
+      <c r="D18" s="211"/>
+      <c r="E18" s="211"/>
+      <c r="F18" s="212"/>
       <c r="G18" s="195"/>
       <c r="H18" s="194"/>
     </row>
@@ -8633,16 +8631,16 @@
       <c r="C19" s="197" t="s">
         <v>96</v>
       </c>
-      <c r="D19" s="206" t="s">
+      <c r="D19" s="204" t="s">
         <v>308</v>
       </c>
-      <c r="E19" s="206" t="s">
+      <c r="E19" s="204" t="s">
         <v>166</v>
       </c>
-      <c r="F19" s="207" t="s">
+      <c r="F19" s="205" t="s">
         <v>325</v>
       </c>
-      <c r="G19" s="208">
+      <c r="G19" s="206">
         <v>2</v>
       </c>
       <c r="H19" s="200">
@@ -8651,56 +8649,56 @@
       </c>
     </row>
     <row r="20" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B20" s="211" t="s">
+      <c r="B20" s="210" t="s">
         <v>319</v>
       </c>
-      <c r="C20" s="212"/>
-      <c r="D20" s="212"/>
-      <c r="E20" s="212"/>
-      <c r="F20" s="213"/>
+      <c r="C20" s="211"/>
+      <c r="D20" s="211"/>
+      <c r="E20" s="211"/>
+      <c r="F20" s="212"/>
       <c r="G20" s="135"/>
       <c r="H20" s="143"/>
     </row>
-    <row r="21" spans="2:8" s="202" customFormat="1" x14ac:dyDescent="0.2">
-      <c r="B21" s="203" t="s">
+    <row r="21" spans="2:8" s="201" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="B21" s="196" t="s">
         <v>140</v>
       </c>
-      <c r="C21" s="167" t="s">
+      <c r="C21" s="197" t="s">
         <v>326</v>
       </c>
-      <c r="D21" s="167">
+      <c r="D21" s="197">
         <v>0.96</v>
       </c>
-      <c r="E21" s="167">
+      <c r="E21" s="197">
         <v>0.9</v>
       </c>
-      <c r="F21" s="224" t="s">
+      <c r="F21" s="305" t="s">
         <v>328</v>
       </c>
-      <c r="G21" s="220">
+      <c r="G21" s="213">
         <v>2</v>
       </c>
-      <c r="H21" s="222">
+      <c r="H21" s="219">
         <f>H19*G21</f>
         <v>144</v>
       </c>
     </row>
-    <row r="22" spans="2:8" s="202" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B22" s="209" t="s">
+    <row r="22" spans="2:8" s="201" customFormat="1" ht="17" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B22" s="306" t="s">
         <v>140</v>
       </c>
-      <c r="C22" s="210" t="s">
+      <c r="C22" s="307" t="s">
         <v>320</v>
       </c>
-      <c r="D22" s="210">
+      <c r="D22" s="307">
         <v>0.7</v>
       </c>
-      <c r="E22" s="210">
+      <c r="E22" s="307">
         <v>0.85</v>
       </c>
-      <c r="F22" s="225"/>
-      <c r="G22" s="221"/>
-      <c r="H22" s="223"/>
+      <c r="F22" s="308"/>
+      <c r="G22" s="309"/>
+      <c r="H22" s="310"/>
     </row>
     <row r="23" spans="2:8" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="B23" s="8"/>
@@ -8740,46 +8738,46 @@
       <c r="H25" s="8"/>
     </row>
     <row r="27" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="C27" s="219" t="s">
+      <c r="C27" s="214" t="s">
         <v>296</v>
       </c>
-      <c r="D27" s="219"/>
-      <c r="E27" s="219"/>
-      <c r="F27" s="219"/>
-      <c r="G27" s="219"/>
+      <c r="D27" s="214"/>
+      <c r="E27" s="214"/>
+      <c r="F27" s="214"/>
+      <c r="G27" s="214"/>
     </row>
     <row r="28" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="C28" s="219"/>
-      <c r="D28" s="219"/>
-      <c r="E28" s="219"/>
-      <c r="F28" s="219"/>
-      <c r="G28" s="219"/>
+      <c r="C28" s="214"/>
+      <c r="D28" s="214"/>
+      <c r="E28" s="214"/>
+      <c r="F28" s="214"/>
+      <c r="G28" s="214"/>
     </row>
     <row r="29" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="C29" s="219"/>
-      <c r="D29" s="219"/>
-      <c r="E29" s="219"/>
-      <c r="F29" s="219"/>
-      <c r="G29" s="219"/>
+      <c r="C29" s="214"/>
+      <c r="D29" s="214"/>
+      <c r="E29" s="214"/>
+      <c r="F29" s="214"/>
+      <c r="G29" s="214"/>
     </row>
   </sheetData>
   <mergeCells count="16">
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B3:F3"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="B14:F14"/>
-    <mergeCell ref="G8:G13"/>
-    <mergeCell ref="C27:G29"/>
-    <mergeCell ref="B20:F20"/>
-    <mergeCell ref="G21:G22"/>
-    <mergeCell ref="H21:H22"/>
-    <mergeCell ref="F21:F22"/>
     <mergeCell ref="B18:F18"/>
     <mergeCell ref="F15:F17"/>
     <mergeCell ref="G15:G17"/>
     <mergeCell ref="H15:H17"/>
     <mergeCell ref="F8:F13"/>
     <mergeCell ref="H8:H13"/>
+    <mergeCell ref="C27:G29"/>
+    <mergeCell ref="B20:F20"/>
+    <mergeCell ref="G21:G22"/>
+    <mergeCell ref="H21:H22"/>
+    <mergeCell ref="F21:F22"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B3:F3"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B14:F14"/>
+    <mergeCell ref="G8:G13"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>

</xml_diff>